<commit_message>
cn-#14 Totally ignore commented line inside of or right after a table.
</commit_message>
<xml_diff>
--- a/test/Cactus.ExcelConverterTest/Features/ConverterTests.xlsx
+++ b/test/Cactus.ExcelConverterTest/Features/ConverterTests.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\itu\Cactus.net\test\Cactus.ExcelConverterTest\Features\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{882BA512-D8BC-4C81-A016-E5E36BD833CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0156D2BB-87F3-4947-B94E-0F88AF5F9770}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-2985" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Exactly Matches" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" iterateCount="250" iterateDelta="1.0000000000000001E-5"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
   <si>
     <t>Given</t>
   </si>
@@ -117,6 +117,12 @@
   </si>
   <si>
     <t>except empty lines</t>
+  </si>
+  <si>
+    <t>Data Grid w commented line</t>
+  </si>
+  <si>
+    <t>DataGridCommentedLine.xlsx</t>
   </si>
 </sst>
 </file>
@@ -434,7 +440,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:E13"/>
+  <dimension ref="A2:E14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.85546875" bestFit="1" customWidth="1"/>
@@ -571,12 +577,28 @@
         <v>25</v>
       </c>
       <c r="D13" t="str">
-        <f t="shared" ref="D13" si="2">SUBSTITUTE(C13, ".xlsx", ".feature")</f>
+        <f t="shared" ref="D13:D14" si="2">SUBSTITUTE(C13, ".xlsx", ".feature")</f>
         <v>FormulaTest.feature</v>
       </c>
       <c r="E13" t="str">
-        <f t="shared" ref="E13" si="3">SUBSTITUTE(C13, ".xlsx", ".exp")</f>
+        <f t="shared" ref="E13:E14" si="3">SUBSTITUTE(C13, ".xlsx", ".exp")</f>
         <v>FormulaTest.exp</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B14" t="s">
+        <v>27</v>
+      </c>
+      <c r="C14" t="s">
+        <v>28</v>
+      </c>
+      <c r="D14" t="str">
+        <f t="shared" si="2"/>
+        <v>DataGridCommentedLine.feature</v>
+      </c>
+      <c r="E14" t="str">
+        <f t="shared" si="3"/>
+        <v>DataGridCommentedLine.exp</v>
       </c>
     </row>
   </sheetData>

</xml_diff>